<commit_message>
Torpedo sinking skip, gun/move broadside priority, savo scenario fix
- Torpedo AI skips already-sunk targets instead of wasting shots
- Remove gun skip for US (no torpedo conservation), JP DD-only skip at ≤3 hex
- Show "撃沈" in fleet status panel for sunk ships (ijn + pf)
- Broadside priority: +3 score penalty for non-broadside targets in gun AI
- AI movement prefers broadside positioning (diagonal approach, lateral when close)
- Strengthen isLineBlocked: check both hexes at hex boundary for torpedo LOS
- Fix savo.html: correct to Battle of Cape Esperance (Oct 11, 1942)
- Add ai_data_africa.json to gitignore (exceeds GitHub 100MB limit)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tanks+/tanks_counters.xlsx
+++ b/tanks+/tanks_counters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/baron/Desktop/aigame/tanks+/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{009E914D-9310-5347-9086-FE8670BFFC65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C63ACF8-81E0-7549-8A1C-C4A6F8C27DF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-31820" yWindow="1880" windowWidth="24980" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="24980" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="US Army" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="50">
   <si>
     <t>M4A1</t>
   </si>
@@ -114,12 +114,6 @@
     <phoneticPr fontId="3"/>
   </si>
   <si>
-    <t>Pz III/I</t>
-  </si>
-  <si>
-    <t>Pz III/I (late)</t>
-  </si>
-  <si>
     <t>Pz IV/H</t>
   </si>
   <si>
@@ -188,9 +182,6 @@
     <t>KV-1C</t>
   </si>
   <si>
-    <t>Su-85</t>
-  </si>
-  <si>
     <t>Su-100</t>
   </si>
   <si>
@@ -198,6 +189,25 @@
   </si>
   <si>
     <t>soviet</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>Pz III/J</t>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Tiger </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="MS Gothic"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>Ⅱ</t>
+    </r>
     <phoneticPr fontId="3"/>
   </si>
 </sst>
@@ -205,7 +215,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -240,8 +250,14 @@
       <family val="2"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="MS Gothic"/>
+      <family val="2"/>
+      <charset val="128"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -261,6 +277,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF8B0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -291,7 +313,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -310,6 +332,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -614,7 +639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -623,7 +648,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>15</v>
@@ -655,7 +680,7 @@
         <v>8</v>
       </c>
       <c r="E2" s="3"/>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -673,7 +698,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="3"/>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -691,7 +716,7 @@
         <v>9</v>
       </c>
       <c r="E4" s="3"/>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -700,16 +725,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C5" s="3">
+        <v>5</v>
+      </c>
+      <c r="D5" s="3">
         <v>7</v>
       </c>
-      <c r="D5" s="3">
-        <v>5</v>
-      </c>
       <c r="E5" s="3"/>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -727,7 +752,7 @@
         <v>7</v>
       </c>
       <c r="E6" s="3"/>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -736,16 +761,16 @@
         <v>5</v>
       </c>
       <c r="B7" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C7" s="3">
+        <v>4</v>
+      </c>
+      <c r="D7" s="3">
         <v>7</v>
       </c>
-      <c r="D7" s="3">
-        <v>5</v>
-      </c>
       <c r="E7" s="3"/>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -763,7 +788,9 @@
         <v>18</v>
       </c>
       <c r="E8" s="3"/>
-      <c r="F8" s="5"/>
+      <c r="F8" s="8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="2" t="s">
@@ -781,7 +808,7 @@
       <c r="E9" s="3">
         <v>1</v>
       </c>
-      <c r="F9" s="5"/>
+      <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
@@ -817,7 +844,7 @@
         <v>7</v>
       </c>
       <c r="E11" s="3"/>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -835,7 +862,7 @@
         <v>8</v>
       </c>
       <c r="E12" s="3"/>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -847,13 +874,13 @@
         <v>6</v>
       </c>
       <c r="C13" s="3">
+        <v>2</v>
+      </c>
+      <c r="D13" s="3">
         <v>9</v>
       </c>
-      <c r="D13" s="3">
-        <v>2</v>
-      </c>
       <c r="E13" s="3"/>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -865,13 +892,13 @@
         <v>6</v>
       </c>
       <c r="C14" s="3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D14" s="3">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E14" s="3"/>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -883,13 +910,13 @@
         <v>6</v>
       </c>
       <c r="C15" s="3">
+        <v>3</v>
+      </c>
+      <c r="D15" s="3">
         <v>9</v>
       </c>
-      <c r="D15" s="3">
-        <v>3</v>
-      </c>
       <c r="E15" s="3"/>
-      <c r="F15" s="5" t="s">
+      <c r="F15" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -907,7 +934,7 @@
         <v>7</v>
       </c>
       <c r="E16" s="3"/>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -916,18 +943,18 @@
         <v>14</v>
       </c>
       <c r="B17" s="3">
+        <v>2</v>
+      </c>
+      <c r="C17" s="3">
         <v>3</v>
       </c>
-      <c r="C17" s="3">
+      <c r="D17" s="3">
         <v>7</v>
-      </c>
-      <c r="D17" s="3">
-        <v>4</v>
       </c>
       <c r="E17" s="3">
         <v>1</v>
       </c>
-      <c r="F17" s="5"/>
+      <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="2" t="s">
@@ -942,10 +969,10 @@
       <c r="D18" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E18" s="3">
-        <v>1</v>
-      </c>
-      <c r="F18" s="5"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="2"/>
@@ -957,7 +984,7 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>15</v>
@@ -977,97 +1004,97 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="2" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="B21" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C21" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D21" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E21" s="3"/>
-      <c r="F21" s="5" t="s">
+      <c r="F21" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" s="3">
         <v>4</v>
       </c>
       <c r="C22" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" s="3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E22" s="3"/>
-      <c r="F22" s="5" t="s">
+      <c r="F22" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B23" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C23" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D23" s="3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E23" s="3"/>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24" s="3">
         <v>6</v>
       </c>
       <c r="C24" s="3">
+        <v>3</v>
+      </c>
+      <c r="D24" s="3">
         <v>9</v>
       </c>
-      <c r="D24" s="3">
-        <v>3</v>
-      </c>
       <c r="E24" s="3"/>
-      <c r="F24" s="5" t="s">
+      <c r="F24" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="2" t="s">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="B25" s="3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C25" s="3">
+        <v>3</v>
+      </c>
+      <c r="D25" s="3">
         <v>9</v>
       </c>
-      <c r="D25" s="3">
-        <v>3</v>
-      </c>
       <c r="E25" s="3"/>
-      <c r="F25" s="5" t="s">
+      <c r="F25" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B26" s="3">
         <v>4</v>
@@ -1078,12 +1105,14 @@
       <c r="D26" s="3">
         <v>8</v>
       </c>
-      <c r="E26" s="3"/>
-      <c r="F26" s="5"/>
+      <c r="E26" s="3">
+        <v>1</v>
+      </c>
+      <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B27" s="3">
         <v>5</v>
@@ -1094,12 +1123,14 @@
       <c r="D27" s="3">
         <v>8</v>
       </c>
-      <c r="E27" s="3"/>
-      <c r="F27" s="5"/>
+      <c r="E27" s="3">
+        <v>1</v>
+      </c>
+      <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B28" s="3">
         <v>4</v>
@@ -1110,14 +1141,14 @@
       <c r="D28" s="3">
         <v>8</v>
       </c>
-      <c r="E28" s="3"/>
-      <c r="F28" s="5">
+      <c r="E28" s="3">
         <v>1</v>
       </c>
+      <c r="F28" s="8"/>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B29" s="3">
         <v>8</v>
@@ -1129,27 +1160,27 @@
         <v>9</v>
       </c>
       <c r="E29" s="3"/>
-      <c r="F29" s="5"/>
+      <c r="F29" s="8"/>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B30" s="3">
         <v>10</v>
       </c>
       <c r="C30" s="3">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D30" s="3">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E30" s="3"/>
-      <c r="F30" s="5"/>
+      <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B31" s="3">
         <v>6</v>
@@ -1161,14 +1192,14 @@
         <v>9</v>
       </c>
       <c r="E31" s="3"/>
-      <c r="F31" s="5"/>
+      <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B32" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C32" s="3">
         <v>4</v>
@@ -1177,29 +1208,29 @@
         <v>8</v>
       </c>
       <c r="E32" s="3"/>
-      <c r="F32" s="5">
-        <v>1</v>
-      </c>
+      <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B33" s="3">
-        <v>4</v>
+        <v>33</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="C33" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D33" s="3">
-        <v>8</v>
-      </c>
-      <c r="E33" s="3"/>
-      <c r="F33" s="5"/>
+        <v>9</v>
+      </c>
+      <c r="E33" s="3">
+        <v>1</v>
+      </c>
+      <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>18</v>
@@ -1208,16 +1239,16 @@
         <v>0</v>
       </c>
       <c r="D34" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E34" s="3">
         <v>1</v>
       </c>
-      <c r="F34" s="5"/>
+      <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>18</v>
@@ -1226,16 +1257,16 @@
         <v>0</v>
       </c>
       <c r="D35" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E35" s="3">
         <v>1</v>
       </c>
-      <c r="F35" s="5"/>
+      <c r="F35" s="8"/>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>18</v>
@@ -1244,240 +1275,210 @@
         <v>0</v>
       </c>
       <c r="D36" s="3">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E36" s="3">
         <v>1</v>
       </c>
-      <c r="F36" s="5"/>
+      <c r="F36" s="8"/>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="2" t="s">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>18</v>
       </c>
       <c r="C37" s="3">
-        <v>0</v>
-      </c>
-      <c r="D37" s="3">
-        <v>9</v>
-      </c>
-      <c r="E37" s="3">
-        <v>1</v>
-      </c>
-      <c r="F37" s="5"/>
+        <v>2</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E37" s="3"/>
+      <c r="F37" s="8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>18</v>
+        <v>37</v>
+      </c>
+      <c r="B38" s="3">
+        <v>1</v>
       </c>
       <c r="C38" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E38" s="3"/>
-      <c r="F38" s="5"/>
+      <c r="F38" s="8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="39" spans="1:6">
-      <c r="A39" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B39" s="3">
-        <v>1</v>
-      </c>
-      <c r="C39" s="3">
-        <v>5</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E39" s="3"/>
+      <c r="A39" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>19</v>
+      </c>
       <c r="F39" s="5"/>
     </row>
     <row r="40" spans="1:6">
-      <c r="A40" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="E40" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="F40" s="5"/>
+      <c r="A40" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" s="3">
+        <v>4</v>
+      </c>
+      <c r="C40" s="3">
+        <v>5</v>
+      </c>
+      <c r="D40" s="3">
+        <v>8</v>
+      </c>
+      <c r="E40" s="3"/>
+      <c r="F40" s="8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B41" s="3">
         <v>5</v>
       </c>
       <c r="C41" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D41" s="3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E41" s="3"/>
-      <c r="F41" s="5" t="s">
+      <c r="F41" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B42" s="3">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C42" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D42" s="3">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E42" s="3"/>
-      <c r="F42" s="5" t="s">
+      <c r="F42" s="8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B43" s="3">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C43" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D43" s="3">
-        <v>11</v>
-      </c>
-      <c r="E43" s="3"/>
-      <c r="F43" s="5" t="s">
-        <v>21</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E43" s="3">
+        <v>1</v>
+      </c>
+      <c r="F43" s="8"/>
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B44" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C44" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D44" s="3">
         <v>8</v>
       </c>
-      <c r="E44" s="3">
-        <v>1</v>
-      </c>
-      <c r="F44" s="5"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="8" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B45" s="3">
         <v>5</v>
       </c>
       <c r="C45" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D45" s="3">
-        <v>8</v>
-      </c>
-      <c r="E45" s="3"/>
-      <c r="F45" s="5" t="s">
-        <v>21</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="E45" s="3">
+        <v>1</v>
+      </c>
+      <c r="F45" s="8"/>
     </row>
     <row r="46" spans="1:6">
       <c r="A46" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B46" s="3">
-        <v>5</v>
+        <v>46</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="C46" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D46" s="3">
-        <v>9</v>
-      </c>
-      <c r="E46" s="3"/>
-      <c r="F46" s="5" t="s">
-        <v>21</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E46" s="3">
+        <v>1</v>
+      </c>
+      <c r="F46" s="8"/>
     </row>
     <row r="47" spans="1:6">
       <c r="A47" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B47" s="3">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="C47" s="3">
-        <v>10</v>
-      </c>
-      <c r="D47" s="3">
-        <v>5</v>
-      </c>
-      <c r="E47" s="3">
-        <v>1</v>
-      </c>
-      <c r="F47" s="5"/>
-    </row>
-    <row r="48" spans="1:6">
-      <c r="A48" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B48" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D47" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C48" s="3">
-        <v>0</v>
-      </c>
-      <c r="D48" s="3">
-        <v>8</v>
-      </c>
-      <c r="E48" s="3">
-        <v>1</v>
-      </c>
-      <c r="F48" s="5"/>
-    </row>
-    <row r="49" spans="1:6">
-      <c r="A49" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C49" s="3">
-        <v>2</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E49" s="3"/>
-      <c r="F49" s="5"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="8" t="s">
+        <v>21</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3"/>

</xml_diff>